<commit_message>
Telecaller daily call report
</commit_message>
<xml_diff>
--- a/public/templates/salespulse-lead-template.xlsx
+++ b/public/templates/salespulse-lead-template.xlsx
@@ -15541,7 +15541,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="I2:I5001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Internet research,Google Maps,Website,Facebook,LinkedIn,Existing database,Referral,Website enquiry,WhatsApp enquiry,Marketing campaign,Excel/CSV import,Other"</formula1>
+      <formula1>"Google Search,VisitFlow,Meta Leads,Referral,Website,Other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15735,7 +15735,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Optional. Product of interest — use the same name as in SalesPulse (e.g. Sales CRM).</t>
+          <t>Optional. Product of interest — use the same name as in SalesPulse (e.g. Visit Flow, Marichi Pulse, Guardly).</t>
         </is>
       </c>
     </row>
@@ -15747,7 +15747,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Optional. Pick from the list (Google Maps, Referral, Facebook…).</t>
+          <t>Optional. Pick from the list: Google Search, VisitFlow, Meta Leads, Referral, Website, Other.</t>
         </is>
       </c>
     </row>
@@ -15860,12 +15860,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Sales CRM</t>
+          <t>Visit Flow</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -15921,7 +15921,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Meta Leads</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>

</xml_diff>